<commit_message>
Update ⑤ 関連性ヒント sheet with additional correlation analysis
Added 4 new correlations (sleep quality→next-day RPE with p=0.021,
nutritional balance→next-day RPE, morning condition→fatigue/RPE)
and protein variety deep-dive section covering lunch/dinner separately,
ingredient-level dinner fish effect, and key finding that lunch protein
presence shows the strongest RPE association (diff -0.89).

https://claude.ai/code/session_01JUjvFGRgwYEsHzNt35Vk6q
</commit_message>
<xml_diff>
--- a/TI_選手_フィードバックシート_20260523.xlsx
+++ b/TI_選手_フィードバックシート_20260523.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="26">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -147,8 +147,28 @@
       <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
+    <font/>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00CC0000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -205,8 +225,32 @@
         <fgColor rgb="00F9FBFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+        <bgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+        <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -261,11 +305,57 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border/>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -407,6 +497,37 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3766,10 +3887,10 @@
           <t>（選手記入欄）</t>
         </is>
       </c>
-      <c r="C35" s="23" t="n"/>
-      <c r="D35" s="23" t="n"/>
-      <c r="E35" s="23" t="n"/>
-      <c r="F35" s="23" t="n"/>
+      <c r="C35" s="52" t="n"/>
+      <c r="D35" s="52" t="n"/>
+      <c r="E35" s="52" t="n"/>
+      <c r="F35" s="10" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="B36" s="21" t="inlineStr">
@@ -3784,10 +3905,10 @@
           <t>（選手記入欄）</t>
         </is>
       </c>
-      <c r="C37" s="23" t="n"/>
-      <c r="D37" s="23" t="n"/>
-      <c r="E37" s="23" t="n"/>
-      <c r="F37" s="23" t="n"/>
+      <c r="C37" s="52" t="n"/>
+      <c r="D37" s="52" t="n"/>
+      <c r="E37" s="52" t="n"/>
+      <c r="F37" s="10" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="B38" s="21" t="inlineStr">
@@ -3802,10 +3923,10 @@
           <t>（選手記入欄）</t>
         </is>
       </c>
-      <c r="C39" s="23" t="n"/>
-      <c r="D39" s="23" t="n"/>
-      <c r="E39" s="23" t="n"/>
-      <c r="F39" s="23" t="n"/>
+      <c r="C39" s="52" t="n"/>
+      <c r="D39" s="52" t="n"/>
+      <c r="E39" s="52" t="n"/>
+      <c r="F39" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="32">
@@ -8733,225 +8854,880 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G14"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="10" customHeight="1"/>
-    <row r="2" ht="22" customHeight="1">
-      <c r="B2" s="24" t="inlineStr">
-        <is>
-          <t>行動とパフォーマンスの関連性（関連しそうなものだけピックアップ）</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="20" customHeight="1">
-      <c r="B4" s="9" t="inlineStr">
+    <row r="1" ht="18" customHeight="1">
+      <c r="A1" s="53" t="inlineStr">
+        <is>
+          <t>■ Section A：既存の関連性ヒント（オリジナル5項目）</t>
+        </is>
+      </c>
+      <c r="B1" s="54" t="n"/>
+      <c r="C1" s="54" t="n"/>
+      <c r="D1" s="54" t="n"/>
+      <c r="E1" s="54" t="n"/>
+      <c r="F1" s="54" t="n"/>
+      <c r="G1" s="55" t="n"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="56" t="inlineStr">
         <is>
           <t>観点</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>A群条件</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>A群平均</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>B群条件</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>B群平均</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="B2" s="56" t="inlineStr">
+        <is>
+          <t>条件A（低/良）</t>
+        </is>
+      </c>
+      <c r="C2" s="56" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D2" s="56" t="inlineStr">
+        <is>
+          <t>条件B（高/悪）</t>
+        </is>
+      </c>
+      <c r="E2" s="56" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="F2" s="56" t="inlineStr">
         <is>
           <t>差(B-A)</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="44" t="inlineStr">
-        <is>
-          <t>練習後補食 vs 翌日の運動後疲労</t>
-        </is>
-      </c>
-      <c r="C5" s="44" t="inlineStr">
-        <is>
-          <t>補食「いいえ」の翌日</t>
-        </is>
-      </c>
-      <c r="D5" s="44" t="n">
-        <v>3.308</v>
-      </c>
-      <c r="E5" s="44" t="inlineStr">
-        <is>
-          <t>補食「はい」の翌日</t>
-        </is>
-      </c>
-      <c r="F5" s="44" t="n">
-        <v>3.645</v>
-      </c>
-      <c r="G5" s="45" t="n">
-        <v>0.337</v>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="44" t="inlineStr">
-        <is>
-          <t>睡眠時間 vs その日のRPE(練習日)</t>
-        </is>
-      </c>
-      <c r="C6" s="44" t="inlineStr">
-        <is>
-          <t>睡眠 &lt; 7時間</t>
-        </is>
-      </c>
-      <c r="D6" s="44" t="n">
-        <v>7.25</v>
-      </c>
-      <c r="E6" s="44" t="inlineStr">
-        <is>
-          <t>睡眠 ≥ 7時間</t>
-        </is>
-      </c>
-      <c r="F6" s="44" t="n">
-        <v>6.216</v>
-      </c>
-      <c r="G6" s="46" t="n">
-        <v>-1.034</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="B7" s="44" t="inlineStr">
-        <is>
-          <t>睡眠の質 vs 運動後疲労(練習日)</t>
-        </is>
-      </c>
-      <c r="C7" s="44" t="inlineStr">
-        <is>
-          <t>睡眠の質 ≥ 3(良くない日)</t>
-        </is>
-      </c>
-      <c r="D7" s="44" t="n">
-        <v>3.524</v>
-      </c>
-      <c r="E7" s="44" t="inlineStr">
-        <is>
-          <t>睡眠の質 ≤ 2</t>
-        </is>
-      </c>
-      <c r="F7" s="44" t="n">
-        <v>3.583</v>
-      </c>
-      <c r="G7" s="45" t="n">
-        <v>0.06</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="B8" s="44" t="inlineStr">
-        <is>
-          <t>水分量 vs 運動後疲労(練習日)</t>
-        </is>
-      </c>
-      <c r="C8" s="44" t="inlineStr">
-        <is>
-          <t>水分 &lt; 1000ml</t>
-        </is>
-      </c>
-      <c r="D8" s="44" t="n">
-        <v>3.125</v>
-      </c>
-      <c r="E8" s="44" t="inlineStr">
-        <is>
-          <t>水分 ≥ 1000ml</t>
-        </is>
-      </c>
-      <c r="F8" s="44" t="n">
-        <v>3.649</v>
-      </c>
-      <c r="G8" s="46" t="n">
-        <v>0.524</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="B9" s="44" t="inlineStr">
-        <is>
-          <t>食材の豊富さ vs 翌日のRPE(練習日)</t>
-        </is>
-      </c>
-      <c r="C9" s="44" t="inlineStr">
-        <is>
-          <t>1〜2種類</t>
-        </is>
-      </c>
-      <c r="D9" s="44" t="n">
-        <v>6.625</v>
-      </c>
-      <c r="E9" s="44" t="inlineStr">
-        <is>
-          <t>3種類以上</t>
-        </is>
-      </c>
-      <c r="F9" s="44" t="n">
-        <v>6.1</v>
-      </c>
-      <c r="G9" s="46" t="n">
-        <v>-0.525</v>
-      </c>
-    </row>
-    <row r="10" ht="10" customHeight="1"/>
-    <row r="11" ht="22" customHeight="1">
-      <c r="B11" s="47" t="inlineStr">
-        <is>
-          <t>■ 読み方のヒント</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="B12" s="48" t="inlineStr">
-        <is>
-          <t>・「差」の絶対値が大きい行ほど、その行動の影響が出ているサイン。0.5以上なら傾向として注目に値する。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="48" t="inlineStr">
-        <is>
-          <t>・練習日のみの平均で比較しています。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="B14" s="48" t="inlineStr">
-        <is>
-          <t>・サンプル数が少ない場合は参考程度に留め、継続データ蓄積で精度が上がります。</t>
-        </is>
-      </c>
-    </row>
+      <c r="G2" s="56" t="inlineStr">
+        <is>
+          <t>注目度</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="57" t="inlineStr">
+        <is>
+          <t>補食(はい/いいえ) → 翌日 運動後疲労</t>
+        </is>
+      </c>
+      <c r="B3" s="58" t="inlineStr">
+        <is>
+          <t>はい: 3.61</t>
+        </is>
+      </c>
+      <c r="C3" s="58" t="n">
+        <v>28</v>
+      </c>
+      <c r="D3" s="58" t="inlineStr">
+        <is>
+          <t>いいえ: 3.44</t>
+        </is>
+      </c>
+      <c r="E3" s="58" t="n">
+        <v>16</v>
+      </c>
+      <c r="F3" s="58" t="n">
+        <v>-0.17</v>
+      </c>
+      <c r="G3" s="58" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="59" t="inlineStr">
+        <is>
+          <t>睡眠時間(≥7h / &lt;7h) → 同日 RPE</t>
+        </is>
+      </c>
+      <c r="B4" s="60" t="inlineStr">
+        <is>
+          <t>≥7h: 6.22</t>
+        </is>
+      </c>
+      <c r="C4" s="60" t="n">
+        <v>37</v>
+      </c>
+      <c r="D4" s="60" t="inlineStr">
+        <is>
+          <t>&lt;7h: 7.25</t>
+        </is>
+      </c>
+      <c r="E4" s="60" t="n">
+        <v>8</v>
+      </c>
+      <c r="F4" s="60" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="G4" s="60" t="inlineStr">
+        <is>
+          <t>★要注目</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="57" t="inlineStr">
+        <is>
+          <t>睡眠の質(良≤2 / 悪≥3) → 同日 運動後疲労</t>
+        </is>
+      </c>
+      <c r="B5" s="58" t="inlineStr">
+        <is>
+          <t>≤2(良): 3.58</t>
+        </is>
+      </c>
+      <c r="C5" s="58" t="n">
+        <v>24</v>
+      </c>
+      <c r="D5" s="58" t="inlineStr">
+        <is>
+          <t>≥3(悪): 3.52</t>
+        </is>
+      </c>
+      <c r="E5" s="58" t="n">
+        <v>21</v>
+      </c>
+      <c r="F5" s="58" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="G5" s="58" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="59" t="inlineStr">
+        <is>
+          <t>水分摂取量(≥1000ml / &lt;1000ml) → 同日 運動後疲労</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>≥1000ml: 3.65</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="n">
+        <v>37</v>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
+        <is>
+          <t>&lt;1000ml: 3.12</t>
+        </is>
+      </c>
+      <c r="E6" s="60" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" s="60" t="n">
+        <v>-0.52</v>
+      </c>
+      <c r="G6" s="60" t="inlineStr">
+        <is>
+          <t>★要注目</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="59" t="inlineStr">
+        <is>
+          <t>タンパク質合計種類数(1〜2種 / 3種以上) → 翌日 RPE</t>
+        </is>
+      </c>
+      <c r="B7" s="60" t="inlineStr">
+        <is>
+          <t>1〜2種: 6.62</t>
+        </is>
+      </c>
+      <c r="C7" s="60" t="n">
+        <v>24</v>
+      </c>
+      <c r="D7" s="60" t="inlineStr">
+        <is>
+          <t>3種以上: 6.10</t>
+        </is>
+      </c>
+      <c r="E7" s="60" t="n">
+        <v>20</v>
+      </c>
+      <c r="F7" s="60" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="G7" s="60" t="inlineStr">
+        <is>
+          <t>★要注目</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="61" t="n"/>
+      <c r="B8" s="61" t="n"/>
+      <c r="C8" s="61" t="n"/>
+      <c r="D8" s="61" t="n"/>
+      <c r="E8" s="61" t="n"/>
+      <c r="F8" s="61" t="n"/>
+      <c r="G8" s="61" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="53" t="inlineStr">
+        <is>
+          <t>■ Section B：新たに判明した関連性（追加4項目）</t>
+        </is>
+      </c>
+      <c r="B9" s="54" t="n"/>
+      <c r="C9" s="54" t="n"/>
+      <c r="D9" s="54" t="n"/>
+      <c r="E9" s="54" t="n"/>
+      <c r="F9" s="54" t="n"/>
+      <c r="G9" s="55" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="56" t="inlineStr">
+        <is>
+          <t>観点</t>
+        </is>
+      </c>
+      <c r="B10" s="56" t="inlineStr">
+        <is>
+          <t>条件A（低/良）</t>
+        </is>
+      </c>
+      <c r="C10" s="56" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D10" s="56" t="inlineStr">
+        <is>
+          <t>条件B（高/悪）</t>
+        </is>
+      </c>
+      <c r="E10" s="56" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="F10" s="56" t="inlineStr">
+        <is>
+          <t>差(B-A)</t>
+        </is>
+      </c>
+      <c r="G10" s="56" t="inlineStr">
+        <is>
+          <t>注目度</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="59" t="inlineStr">
+        <is>
+          <t>睡眠の質(良好≤2 / 不良≥3) → 翌日 RPE  ★統計的有意(p=0.021)</t>
+        </is>
+      </c>
+      <c r="B11" s="60" t="inlineStr">
+        <is>
+          <t>良好≤2: 6.69</t>
+        </is>
+      </c>
+      <c r="C11" s="60" t="n">
+        <v>26</v>
+      </c>
+      <c r="D11" s="60" t="inlineStr">
+        <is>
+          <t>不良≥3: 5.94</t>
+        </is>
+      </c>
+      <c r="E11" s="60" t="n">
+        <v>18</v>
+      </c>
+      <c r="F11" s="60" t="n">
+        <v>-0.75</v>
+      </c>
+      <c r="G11" s="60" t="inlineStr">
+        <is>
+          <t>★要注目</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="59" t="inlineStr">
+        <is>
+          <t>栄養バランス(良好1〜2 / 不良3〜4) → 翌日 RPE</t>
+        </is>
+      </c>
+      <c r="B12" s="60" t="inlineStr">
+        <is>
+          <t>良好1〜2: 5.94</t>
+        </is>
+      </c>
+      <c r="C12" s="60" t="n">
+        <v>16</v>
+      </c>
+      <c r="D12" s="60" t="inlineStr">
+        <is>
+          <t>不良3〜4: 6.64</t>
+        </is>
+      </c>
+      <c r="E12" s="60" t="n">
+        <v>28</v>
+      </c>
+      <c r="F12" s="60" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="G12" s="60" t="inlineStr">
+        <is>
+          <t>★要注目</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="59" t="inlineStr">
+        <is>
+          <t>起床時コンディション(良好1〜2 / 不調4〜5) → 同日 運動後疲労</t>
+        </is>
+      </c>
+      <c r="B13" s="60" t="inlineStr">
+        <is>
+          <t>良好1〜2: 3.22</t>
+        </is>
+      </c>
+      <c r="C13" s="60" t="n">
+        <v>18</v>
+      </c>
+      <c r="D13" s="60" t="inlineStr">
+        <is>
+          <t>不調4〜5: 4.00</t>
+        </is>
+      </c>
+      <c r="E13" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="60" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G13" s="60" t="inlineStr">
+        <is>
+          <t>★要注目</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="59" t="inlineStr">
+        <is>
+          <t>起床時コンディション(良好1〜2 / 不調4〜5) → 同日 RPE</t>
+        </is>
+      </c>
+      <c r="B14" s="60" t="inlineStr">
+        <is>
+          <t>良好1〜2: 6.33</t>
+        </is>
+      </c>
+      <c r="C14" s="60" t="n">
+        <v>18</v>
+      </c>
+      <c r="D14" s="60" t="inlineStr">
+        <is>
+          <t>不調4〜5: 5.00</t>
+        </is>
+      </c>
+      <c r="E14" s="60" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="60" t="n">
+        <v>-1.33</v>
+      </c>
+      <c r="G14" s="60" t="inlineStr">
+        <is>
+          <t>★要注目</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1"/>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="53" t="inlineStr">
+        <is>
+          <t>■ Section C：昼食・夕食タンパク質の詳細分析</t>
+        </is>
+      </c>
+      <c r="B16" s="54" t="n"/>
+      <c r="C16" s="54" t="n"/>
+      <c r="D16" s="54" t="n"/>
+      <c r="E16" s="54" t="n"/>
+      <c r="F16" s="54" t="n"/>
+      <c r="G16" s="55" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="62" t="inlineStr">
+        <is>
+          <t>平均タンパク質種類数　昼食: 0.68種 / 夕食: 1.60種</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  昼食タンパク質との関連</t>
+        </is>
+      </c>
+      <c r="B18" s="54" t="n"/>
+      <c r="C18" s="54" t="n"/>
+      <c r="D18" s="54" t="n"/>
+      <c r="E18" s="54" t="n"/>
+      <c r="F18" s="54" t="n"/>
+      <c r="G18" s="55" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="56" t="inlineStr">
+        <is>
+          <t>観点</t>
+        </is>
+      </c>
+      <c r="B19" s="56" t="inlineStr">
+        <is>
+          <t>条件A（低/良）</t>
+        </is>
+      </c>
+      <c r="C19" s="56" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D19" s="56" t="inlineStr">
+        <is>
+          <t>条件B（高/悪）</t>
+        </is>
+      </c>
+      <c r="E19" s="56" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="F19" s="56" t="inlineStr">
+        <is>
+          <t>差(B-A)</t>
+        </is>
+      </c>
+      <c r="G19" s="56" t="inlineStr">
+        <is>
+          <t>注目度</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="59" t="inlineStr">
+        <is>
+          <t>昼食タンパク質種類数(0種 / 1種以上) → 翌日 RPE</t>
+        </is>
+      </c>
+      <c r="B20" s="60" t="inlineStr">
+        <is>
+          <t>0種: 6.89</t>
+        </is>
+      </c>
+      <c r="C20" s="60" t="n">
+        <v>19</v>
+      </c>
+      <c r="D20" s="60" t="inlineStr">
+        <is>
+          <t>1種以上: 6.00</t>
+        </is>
+      </c>
+      <c r="E20" s="60" t="n">
+        <v>25</v>
+      </c>
+      <c r="F20" s="60" t="n">
+        <v>-0.89</v>
+      </c>
+      <c r="G20" s="60" t="inlineStr">
+        <is>
+          <t>★要注目</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="57" t="inlineStr">
+        <is>
+          <t>昼食タンパク質種類数(0種 / 1種以上) → 翌日 運動後疲労</t>
+        </is>
+      </c>
+      <c r="B21" s="58" t="inlineStr">
+        <is>
+          <t>0種: 3.68</t>
+        </is>
+      </c>
+      <c r="C21" s="58" t="n">
+        <v>19</v>
+      </c>
+      <c r="D21" s="58" t="inlineStr">
+        <is>
+          <t>1種以上: 3.44</t>
+        </is>
+      </c>
+      <c r="E21" s="58" t="n">
+        <v>25</v>
+      </c>
+      <c r="F21" s="58" t="n">
+        <v>-0.24</v>
+      </c>
+      <c r="G21" s="58" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1"/>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  夕食タンパク質との関連</t>
+        </is>
+      </c>
+      <c r="B23" s="54" t="n"/>
+      <c r="C23" s="54" t="n"/>
+      <c r="D23" s="54" t="n"/>
+      <c r="E23" s="54" t="n"/>
+      <c r="F23" s="54" t="n"/>
+      <c r="G23" s="55" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="56" t="inlineStr">
+        <is>
+          <t>観点</t>
+        </is>
+      </c>
+      <c r="B24" s="56" t="inlineStr">
+        <is>
+          <t>条件A（低/良）</t>
+        </is>
+      </c>
+      <c r="C24" s="56" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D24" s="56" t="inlineStr">
+        <is>
+          <t>条件B（高/悪）</t>
+        </is>
+      </c>
+      <c r="E24" s="56" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="F24" s="56" t="inlineStr">
+        <is>
+          <t>差(B-A)</t>
+        </is>
+      </c>
+      <c r="G24" s="56" t="inlineStr">
+        <is>
+          <t>注目度</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="59" t="inlineStr">
+        <is>
+          <t>夕食タンパク質種類数(1〜2種 / 3種以上) → 翌日 RPE</t>
+        </is>
+      </c>
+      <c r="B25" s="60" t="inlineStr">
+        <is>
+          <t>1〜2種: 6.52</t>
+        </is>
+      </c>
+      <c r="C25" s="60" t="n">
+        <v>33</v>
+      </c>
+      <c r="D25" s="60" t="inlineStr">
+        <is>
+          <t>3種以上: 6.00</t>
+        </is>
+      </c>
+      <c r="E25" s="60" t="n">
+        <v>11</v>
+      </c>
+      <c r="F25" s="60" t="n">
+        <v>-0.52</v>
+      </c>
+      <c r="G25" s="60" t="inlineStr">
+        <is>
+          <t>★要注目</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="57" t="inlineStr">
+        <is>
+          <t>夕食タンパク質種類数(1〜2種 / 3種以上) → 翌日 運動後疲労</t>
+        </is>
+      </c>
+      <c r="B26" s="58" t="inlineStr">
+        <is>
+          <t>1〜2種: 3.55</t>
+        </is>
+      </c>
+      <c r="C26" s="58" t="n">
+        <v>33</v>
+      </c>
+      <c r="D26" s="58" t="inlineStr">
+        <is>
+          <t>3種以上: 3.55</t>
+        </is>
+      </c>
+      <c r="E26" s="58" t="n">
+        <v>11</v>
+      </c>
+      <c r="F26" s="58" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="58" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="57" t="inlineStr">
+        <is>
+          <t>夕食タンパク質種類数(1〜2種 / 3種以上) → 翌日 起床時コンディション</t>
+        </is>
+      </c>
+      <c r="B27" s="58" t="inlineStr">
+        <is>
+          <t>1〜2種: 2.56</t>
+        </is>
+      </c>
+      <c r="C27" s="58" t="n">
+        <v>41</v>
+      </c>
+      <c r="D27" s="58" t="inlineStr">
+        <is>
+          <t>3種以上: 2.64</t>
+        </is>
+      </c>
+      <c r="E27" s="58" t="n">
+        <v>11</v>
+      </c>
+      <c r="F27" s="58" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="G27" s="58" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1"/>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  食材別（夕食）との関連 → 翌日 RPE</t>
+        </is>
+      </c>
+      <c r="B29" s="54" t="n"/>
+      <c r="C29" s="54" t="n"/>
+      <c r="D29" s="54" t="n"/>
+      <c r="E29" s="54" t="n"/>
+      <c r="F29" s="54" t="n"/>
+      <c r="G29" s="55" t="n"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="56" t="inlineStr">
+        <is>
+          <t>観点</t>
+        </is>
+      </c>
+      <c r="B30" s="56" t="inlineStr">
+        <is>
+          <t>条件A（低/良）</t>
+        </is>
+      </c>
+      <c r="C30" s="56" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="D30" s="56" t="inlineStr">
+        <is>
+          <t>条件B（高/悪）</t>
+        </is>
+      </c>
+      <c r="E30" s="56" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="F30" s="56" t="inlineStr">
+        <is>
+          <t>差(B-A)</t>
+        </is>
+      </c>
+      <c r="G30" s="56" t="inlineStr">
+        <is>
+          <t>注目度</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="59" t="inlineStr">
+        <is>
+          <t>夕食に魚(なし / あり) → 翌日 RPE</t>
+        </is>
+      </c>
+      <c r="B31" s="60" t="inlineStr">
+        <is>
+          <t>なし: 6.62</t>
+        </is>
+      </c>
+      <c r="C31" s="60" t="n">
+        <v>24</v>
+      </c>
+      <c r="D31" s="60" t="inlineStr">
+        <is>
+          <t>あり: 6.10</t>
+        </is>
+      </c>
+      <c r="E31" s="60" t="n">
+        <v>20</v>
+      </c>
+      <c r="F31" s="60" t="n">
+        <v>-0.53</v>
+      </c>
+      <c r="G31" s="60" t="inlineStr">
+        <is>
+          <t>★要注目</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="57" t="inlineStr">
+        <is>
+          <t>夕食に肉(なし / あり) → 翌日 RPE</t>
+        </is>
+      </c>
+      <c r="B32" s="58" t="inlineStr">
+        <is>
+          <t>なし: 6.47</t>
+        </is>
+      </c>
+      <c r="C32" s="58" t="n">
+        <v>15</v>
+      </c>
+      <c r="D32" s="58" t="inlineStr">
+        <is>
+          <t>あり: 6.34</t>
+        </is>
+      </c>
+      <c r="E32" s="58" t="n">
+        <v>29</v>
+      </c>
+      <c r="F32" s="58" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="G32" s="58" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="57" t="inlineStr">
+        <is>
+          <t>夕食に豆(なし / あり) → 翌日 RPE</t>
+        </is>
+      </c>
+      <c r="B33" s="58" t="inlineStr">
+        <is>
+          <t>なし: 6.39</t>
+        </is>
+      </c>
+      <c r="C33" s="58" t="n">
+        <v>31</v>
+      </c>
+      <c r="D33" s="58" t="inlineStr">
+        <is>
+          <t>あり: 6.38</t>
+        </is>
+      </c>
+      <c r="E33" s="58" t="n">
+        <v>13</v>
+      </c>
+      <c r="F33" s="58" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="G33" s="58" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="57" t="inlineStr">
+        <is>
+          <t>夕食に卵(なし / あり) → 翌日 RPE</t>
+        </is>
+      </c>
+      <c r="B34" s="58" t="inlineStr">
+        <is>
+          <t>なし: 6.44</t>
+        </is>
+      </c>
+      <c r="C34" s="58" t="n">
+        <v>32</v>
+      </c>
+      <c r="D34" s="58" t="inlineStr">
+        <is>
+          <t>あり: 6.25</t>
+        </is>
+      </c>
+      <c r="E34" s="58" t="n">
+        <v>12</v>
+      </c>
+      <c r="F34" s="58" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="G34" s="58" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1"/>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="64" t="inlineStr">
+        <is>
+          <t>※ 差の絶対値 0.5以上→要注目（黄色）、0.3以上→参考（薄黄色）</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1"/>
+    <row r="38" ht="18" customHeight="1"/>
+    <row r="39" ht="18" customHeight="1"/>
+    <row r="40" ht="18" customHeight="1"/>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="B2:G2"/>
-    <mergeCell ref="B14:G14"/>
-    <mergeCell ref="B12:G12"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="B11:G11"/>
+  <mergeCells count="8">
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>